<commit_message>
Recompute sensitivity analyses with final 15-expert weights
</commit_message>
<xml_diff>
--- a/data/platform_score_package/lcdp_skill_burden_calculations.xlsx
+++ b/data/platform_score_package/lcdp_skill_burden_calculations.xlsx
@@ -12,6 +12,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Final_Ranking" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weight_Set_Check" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase8I_Ablation_Diagnostic" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sens_Skill_Final15" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sens_Skill_Summary15" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sens_Phase_Final15" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sens_Aggregation15" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Switching_Final15" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -514,6 +519,338 @@
         <is>
           <t>Previous sensitivity and switching-point sheets based on the older weight set were intentionally removed and must be recomputed before being cited.</t>
         </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Final 15-expert sensitivity analyses</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Sensitivity and switching-point outputs were recomputed from the corrected final 15-expert Round 2 consensus weights. The workbook includes Sens_Skill_Final15, Sens_Skill_Summary15, Sens_Phase_Final15, Sens_Aggregation15, and Switching_Final15.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Application Logic diagnostic</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>The skill-weight perturbation diagnostic uses a reproducible keyword-defined Application Logic and Programming subset implemented in analysis/recompute_sensitivity_from_final_weights.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Phase 8I diagnostic</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>The unweighted requirement-count ranking is identical to the weighted Total ISBI ranking, so the ablation diagnostic is retained for reproducibility but is not recommended as a separate manuscript subsection.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Adjacent_Pair</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Total_Gap</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Dominant_Phase_Difference</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Delta_Design</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Delta_Development</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Delta_Implementation</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Boundary_Coeff_Design</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Boundary_Coeff_Development</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Boundary_RHS</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Boundary_Equation</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Average_Skill_Weight</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Resilience_Errors_Ceil</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Aurea vs. Google AppSheet</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>176.7333333333333</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>53.39999999999998</v>
+      </c>
+      <c r="E2" t="n">
+        <v>102.0666666666667</v>
+      </c>
+      <c r="F2" t="n">
+        <v>21.26666666666665</v>
+      </c>
+      <c r="G2" t="n">
+        <v>32.13333333333333</v>
+      </c>
+      <c r="H2" t="n">
+        <v>80.80000000000001</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-21.26666666666665</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>32.13 omega_A + 80.80 omega_D = -21.27</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>10.39872408293461</v>
+      </c>
+      <c r="L2" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Google AppSheet vs. OutSystems</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>32.39999999999998</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>-57.59999999999999</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-14.93333333333331</v>
+      </c>
+      <c r="F3" t="n">
+        <v>104.9333333333333</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-162.5333333333333</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-119.8666666666666</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-104.9333333333333</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>-162.53 omega_A + -119.87 omega_D = -104.93</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>10.39872408293461</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OutSystems vs. Zoho Creator</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>20.86666666666667</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3.066666666666677</v>
+      </c>
+      <c r="E4" t="n">
+        <v>37.73333333333329</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-19.93333333333334</v>
+      </c>
+      <c r="G4" t="n">
+        <v>23.00000000000001</v>
+      </c>
+      <c r="H4" t="n">
+        <v>57.66666666666663</v>
+      </c>
+      <c r="I4" t="n">
+        <v>19.93333333333334</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>23.00 omega_A + 57.67 omega_D = 19.93</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>10.39872408293461</v>
+      </c>
+      <c r="L4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Zoho Creator vs. Microsoft Power Apps</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>30.4666666666667</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Development</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.6000000000000085</v>
+      </c>
+      <c r="E5" t="n">
+        <v>111.1333333333334</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-81.26666666666668</v>
+      </c>
+      <c r="G5" t="n">
+        <v>81.86666666666669</v>
+      </c>
+      <c r="H5" t="n">
+        <v>192.4000000000001</v>
+      </c>
+      <c r="I5" t="n">
+        <v>81.26666666666668</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>81.87 omega_A + 192.40 omega_D = 81.27</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>10.39872408293461</v>
+      </c>
+      <c r="L5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Microsoft Power Apps vs. Mendix</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>156.7333333333333</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Implementation</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>149.6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-191.8</v>
+      </c>
+      <c r="F6" t="n">
+        <v>198.9333333333334</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-49.33333333333337</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-390.7333333333333</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-198.9333333333334</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>-49.33 omega_A + -390.73 omega_D = -198.93</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>10.39872408293461</v>
+      </c>
+      <c r="L6" t="n">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -10934,4 +11271,688 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Base_Rank</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ApplicationLogic_plus20_Rank</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ApplicationLogic_plus20_Change</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ApplicationLogic_minus20_Rank</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ApplicationLogic_minus20_Change</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Aurea</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Google AppSheet</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OutSystems</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Zoho Creator</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Microsoft Power Apps</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mendix</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Application_Logic_Skill_Rows</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Spearman_plus20</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Spearman_minus20</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>First_Rank_Change_Increase_Pct_Approx</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>First_Rank_Change_Decrease_Pct_Approx</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.4200000000000002</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.2900000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Base_Rank</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Equal_Normalized_Rank</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Equal_Normalized_Change</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Development_060_Rank</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Development_060_Change</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Implementation_Deemphasized_010_Rank</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Implementation_Deemphasized_010_Change</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Development_090_Rank</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Development_090_Change</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Aurea</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Google AppSheet</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OutSystems</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Zoho Creator</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Microsoft Power Apps</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>6</v>
+      </c>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mendix</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" t="n">
+        <v>-4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Base_Rank</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>p2_q1_Rank</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>p2_q1_Change</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>p1_qinf_Rank</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>p1_qinf_Change</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Aurea</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Google AppSheet</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>OutSystems</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Zoho Creator</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Microsoft Power Apps</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Mendix</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>